<commit_message>
Publish workbenches for 2026-10-18
</commit_message>
<xml_diff>
--- a/docs/downloads/经营分_山西省区__山西东片区_2026-10-18.xlsx
+++ b/docs/downloads/经营分_山西省区__山西东片区_2026-10-18.xlsx
@@ -1219,33 +1219,33 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>7544177702270404651</t>
+          <t>7044370571840194568</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>IU酒店（太原山大一院迎泽公园店）</t>
+          <t>希岸·轻雅酒店(太原柳巷大南门地铁站店)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>iu酒店(山大一院迎泽公园店)</t>
+          <t>希岸·轻雅酒店(太原柳巷大南门地铁站店)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>已认证</t>
+          <t>未认证</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>稳房源,提质量,附加分,拿收益</t>
+          <t>稳房源,提质量,拿收益</t>
         </is>
       </c>
       <c r="K8" t="n">
@@ -1255,25 +1255,25 @@
         <v>10</v>
       </c>
       <c r="M8" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="N8" t="n">
         <v>30</v>
       </c>
       <c r="O8" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="P8" t="n">
         <v>30</v>
       </c>
       <c r="Q8" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="R8" t="n">
         <v>30</v>
       </c>
       <c r="S8" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="T8" t="n">
         <v>20</v>
@@ -1300,24 +1300,20 @@
           <t>山西东片区</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>太原市</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>7044370571840194568</t>
+          <t>7543445920772278322</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>希岸·轻雅酒店(太原柳巷大南门地铁站店)</t>
+          <t>潮漫酒店（太原火车站服装城五一广场店）</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>希岸·轻雅酒店(太原柳巷大南门地铁站店)</t>
+          <t>潮漫酒店(太原火车站五一广场店)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1329,11 +1325,11 @@
         <v>85</v>
       </c>
       <c r="I9" t="n">
-        <v>-2</v>
+        <v>-5</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>稳房源,提质量,拿收益</t>
+          <t>提质量,拿收益</t>
         </is>
       </c>
       <c r="K9" t="n">
@@ -1343,19 +1339,19 @@
         <v>10</v>
       </c>
       <c r="M9" t="n">
+        <v>30</v>
+      </c>
+      <c r="N9" t="n">
+        <v>30</v>
+      </c>
+      <c r="O9" t="n">
         <v>25</v>
       </c>
-      <c r="N9" t="n">
-        <v>30</v>
-      </c>
-      <c r="O9" t="n">
-        <v>20</v>
-      </c>
       <c r="P9" t="n">
         <v>30</v>
       </c>
       <c r="Q9" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
         <v>30</v>
@@ -1388,36 +1384,40 @@
           <t>山西东片区</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>太原市</t>
+        </is>
+      </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>7543445920772278322</t>
+          <t>7544177702270404651</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>潮漫酒店（太原火车站服装城五一广场店）</t>
+          <t>IU酒店（太原山大一院迎泽公园店）</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>潮漫酒店(太原火车站五一广场店)</t>
+          <t>iu酒店(山大一院迎泽公园店)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>未认证</t>
+          <t>已认证</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I10" t="n">
-        <v>-5</v>
+        <v>7</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>提质量,拿收益</t>
+          <t>稳房源,提质量,附加分,拿收益</t>
         </is>
       </c>
       <c r="K10" t="n">
@@ -1427,7 +1427,7 @@
         <v>10</v>
       </c>
       <c r="M10" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="N10" t="n">
         <v>30</v>
@@ -1439,13 +1439,13 @@
         <v>30</v>
       </c>
       <c r="Q10" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R10" t="n">
         <v>30</v>
       </c>
       <c r="S10" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="T10" t="n">
         <v>20</v>
@@ -1582,7 +1582,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>已认证</t>
+          <t>未认证</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>已认证</t>
+          <t>未认证</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -2022,7 +2022,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>未认证</t>
+          <t>已认证</t>
         </is>
       </c>
       <c r="H17" t="n">
@@ -2095,17 +2095,17 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>6601138073352800270</t>
+          <t>6601139644534884366</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>锦江之星品尚(太原平阳路店)</t>
+          <t>锦江都城酒店（太原茂业天地长风街地铁站店）</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>锦江之星品尚酒店(太原平阳路店)</t>
+          <t>锦江都城酒店(太原长风街地铁站店)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2117,7 +2117,7 @@
         <v>90</v>
       </c>
       <c r="I18" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -2183,29 +2183,29 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>6601139644534884366</t>
+          <t>6601150433513703437</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>锦江都城酒店（太原茂业天地长风街地铁站店）</t>
+          <t>7天酒店（太原火车站服装城省人民医院店）</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>锦江都城酒店(太原长风街地铁站店)</t>
+          <t>7天酒店(太原火车站店)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>已认证</t>
+          <t>未认证</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -2219,7 +2219,7 @@
         <v>10</v>
       </c>
       <c r="M19" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="N19" t="n">
         <v>30</v>
@@ -2231,7 +2231,7 @@
         <v>30</v>
       </c>
       <c r="Q19" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="R19" t="n">
         <v>30</v>
@@ -2271,29 +2271,29 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>6601150433513703437</t>
+          <t>6601138073352800270</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>7天酒店（太原火车站服装城省人民医院店）</t>
+          <t>锦江之星品尚(太原平阳路店)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>7天酒店(太原火车站店)</t>
+          <t>锦江之星品尚酒店(太原平阳路店)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>未认证</t>
+          <t>已认证</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="I20" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -2307,7 +2307,7 @@
         <v>10</v>
       </c>
       <c r="M20" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="N20" t="n">
         <v>30</v>
@@ -2557,7 +2557,7 @@
         <v>100</v>
       </c>
       <c r="I23" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -2623,17 +2623,17 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>6601131638728427523</t>
+          <t>7277051619374532645</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>锦江之星（太原柳巷大南门地铁站迎泽公园酒店）</t>
+          <t>维也纳3好酒店(太原动物园店)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>锦江之星(太原大南门地铁站迎泽公园店)</t>
+          <t>维也纳3好酒店(太原动物园店)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2645,11 +2645,11 @@
         <v>100</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>稳房源,提质量,拿收益</t>
+          <t>提质量,拿收益</t>
         </is>
       </c>
       <c r="K24" t="n">
@@ -2659,19 +2659,19 @@
         <v>10</v>
       </c>
       <c r="M24" t="n">
+        <v>30</v>
+      </c>
+      <c r="N24" t="n">
+        <v>30</v>
+      </c>
+      <c r="O24" t="n">
         <v>25</v>
       </c>
-      <c r="N24" t="n">
-        <v>30</v>
-      </c>
-      <c r="O24" t="n">
-        <v>20</v>
-      </c>
       <c r="P24" t="n">
         <v>30</v>
       </c>
       <c r="Q24" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="R24" t="n">
         <v>30</v>
@@ -2799,17 +2799,17 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>7277051619374532645</t>
+          <t>6601131638728427523</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>维也纳3好酒店(太原动物园店)</t>
+          <t>锦江之星（太原柳巷大南门地铁站迎泽公园酒店）</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>维也纳3好酒店(太原动物园店)</t>
+          <t>锦江之星(太原大南门地铁站迎泽公园店)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2821,11 +2821,11 @@
         <v>105</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>提质量,拿收益</t>
+          <t>稳房源,提质量,拿收益</t>
         </is>
       </c>
       <c r="K26" t="n">
@@ -2835,7 +2835,7 @@
         <v>10</v>
       </c>
       <c r="M26" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="N26" t="n">
         <v>30</v>
@@ -2847,7 +2847,7 @@
         <v>30</v>
       </c>
       <c r="Q26" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="R26" t="n">
         <v>30</v>
@@ -3166,7 +3166,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>已认证</t>
+          <t>未认证</t>
         </is>
       </c>
       <c r="H30" t="n">

</xml_diff>